<commit_message>
WIP - J1939 rx list edited down to whats on the data sheet
</commit_message>
<xml_diff>
--- a/T620X_IO.xlsx
+++ b/T620X_IO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLC_DEV\MTech\Mtech_T620X_Trommel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev_plc\MTech\MTech_T620X_Trommel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0FBAE4-DA39-47A2-9099-4879E8FF8915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85BE2FD-ADBE-493C-9E30-B61AFBF7D8BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="857" activeTab="8" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="857" activeTab="7" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
   </bookViews>
   <sheets>
     <sheet name="IO" sheetId="11" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2617" uniqueCount="1008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3124" uniqueCount="1187">
   <si>
     <t>PLC Name</t>
   </si>
@@ -3073,6 +3073,543 @@
   </si>
   <si>
     <t>UDINT</t>
+  </si>
+  <si>
+    <t>AccelPedal1LowIdleSwitch</t>
+  </si>
+  <si>
+    <t>AccelPedalKickdownSwitch</t>
+  </si>
+  <si>
+    <t>RoadSpeedLimitStatus</t>
+  </si>
+  <si>
+    <t>AccelPedal2LowIdleSwitch</t>
+  </si>
+  <si>
+    <t>AccelPedalPos1</t>
+  </si>
+  <si>
+    <t>EngPercentLoadAtCurrentSpeed</t>
+  </si>
+  <si>
+    <t>RemoteAccelPedalPos</t>
+  </si>
+  <si>
+    <t>AccelPedalPos2</t>
+  </si>
+  <si>
+    <t>VhclAccelerationRateLimitStatus</t>
+  </si>
+  <si>
+    <t>MmntryEngMaxPowerEnableFeedback</t>
+  </si>
+  <si>
+    <t>DPFThermalManagementActive</t>
+  </si>
+  <si>
+    <t>SCRThermalManagementActive</t>
+  </si>
+  <si>
+    <t>ActlMxAvailableEngPercentTorque</t>
+  </si>
+  <si>
+    <t>EstPumpingPercentTorque</t>
+  </si>
+  <si>
+    <t>NominalFrictionPercentTorque</t>
+  </si>
+  <si>
+    <t>EngsDesiredOperatingSpeed</t>
+  </si>
+  <si>
+    <t>EngsDsrdOprtngSpdAsymmtryAdjstmn</t>
+  </si>
+  <si>
+    <t>EstEngPrsticLossesPercentTorque</t>
+  </si>
+  <si>
+    <t>Aftrtratment1ExhaustGasMassFlow</t>
+  </si>
+  <si>
+    <t>Aftertreatment1IntakeDewPoint</t>
+  </si>
+  <si>
+    <t>Aftertreatment1ExhaustDewPoint</t>
+  </si>
+  <si>
+    <t>Aftertreatment2IntakeDewPoint</t>
+  </si>
+  <si>
+    <t>Aftertreatment2ExhaustDewPoint</t>
+  </si>
+  <si>
+    <t>REAl</t>
+  </si>
+  <si>
+    <t>EngTrb1ClcltedTurbineIntakeTemp</t>
+  </si>
+  <si>
+    <t>EngTrb1ClcltedTurbineOutletTemp</t>
+  </si>
+  <si>
+    <t>EngExhstGsRcrculation1ValveCtrl</t>
+  </si>
+  <si>
+    <t>EngVrblGmtryTrbArCtrlShtffValve</t>
+  </si>
+  <si>
+    <t>EngVrableGeometryTurbo1CtrlMode</t>
+  </si>
+  <si>
+    <t>EngVrblGometryTurbo1ActuatorPos</t>
+  </si>
+  <si>
+    <t>EngCoolantTemp</t>
+  </si>
+  <si>
+    <t>EngFuelTemp1</t>
+  </si>
+  <si>
+    <t>EngOilTemp1</t>
+  </si>
+  <si>
+    <t>EngTurboOilTemp</t>
+  </si>
+  <si>
+    <t>EngIntercoolerTemp</t>
+  </si>
+  <si>
+    <t>EngIntercoolerThermostatOpening</t>
+  </si>
+  <si>
+    <t>EngFuelDeliveryPress</t>
+  </si>
+  <si>
+    <t>EngExCrankcaseBlowbyPress</t>
+  </si>
+  <si>
+    <t>EngOilLevel</t>
+  </si>
+  <si>
+    <t>EngOilPress</t>
+  </si>
+  <si>
+    <t>EngCrankcasePress</t>
+  </si>
+  <si>
+    <t>EngCoolantPress</t>
+  </si>
+  <si>
+    <t>EngCoolantLevel</t>
+  </si>
+  <si>
+    <t>UINT</t>
+  </si>
+  <si>
+    <t>EFL_P1</t>
+  </si>
+  <si>
+    <t>EngInjectionCtrlPress</t>
+  </si>
+  <si>
+    <t>EngInjectorMeteringRail1Press</t>
+  </si>
+  <si>
+    <t>EngInjectorTimingRail1Press</t>
+  </si>
+  <si>
+    <t>EngInjectorMeteringRail2Press</t>
+  </si>
+  <si>
+    <t>LREAL</t>
+  </si>
+  <si>
+    <t>EngTripFuel</t>
+  </si>
+  <si>
+    <t>EngTotalFuelUsed</t>
+  </si>
+  <si>
+    <t>BarometricPress</t>
+  </si>
+  <si>
+    <t>CabInteriorTemp</t>
+  </si>
+  <si>
+    <t>AmbientAirTemp</t>
+  </si>
+  <si>
+    <t>EngAirIntakeTemp</t>
+  </si>
+  <si>
+    <t>RoadSurfaceTemp</t>
+  </si>
+  <si>
+    <t>EngDslPrtclateFilterIntakePress</t>
+  </si>
+  <si>
+    <t>EngIntakeManifold1Press</t>
+  </si>
+  <si>
+    <t>EngIntakeManifold1Temp</t>
+  </si>
+  <si>
+    <t>EngAirIntakePress</t>
+  </si>
+  <si>
+    <t>EngAirFilter1DiffPress</t>
+  </si>
+  <si>
+    <t>EngExhaustGasTemp</t>
+  </si>
+  <si>
+    <t>EngCoolantFilterDiffPress</t>
+  </si>
+  <si>
+    <t>IC1</t>
+  </si>
+  <si>
+    <t>NetBatteryCurrent</t>
+  </si>
+  <si>
+    <t>AltCurrent</t>
+  </si>
+  <si>
+    <t>ChargingSystemPotential</t>
+  </si>
+  <si>
+    <t>BatteryPotential_PowerInput1</t>
+  </si>
+  <si>
+    <t>KeyswitchBatteryPotential</t>
+  </si>
+  <si>
+    <t>EngOilLevelRemoteReservoir</t>
+  </si>
+  <si>
+    <t>EngFuelSupplyPumpIntakePress</t>
+  </si>
+  <si>
+    <t>EngFuelFilterDiffPress</t>
+  </si>
+  <si>
+    <t>EngWasteOilReservoirLevel</t>
+  </si>
+  <si>
+    <t>EngOilFilterOutletPress</t>
+  </si>
+  <si>
+    <t>EngOilPrimingPumpSwitch</t>
+  </si>
+  <si>
+    <t>EngOilPrimingState</t>
+  </si>
+  <si>
+    <t>EngOilPreHeatedState</t>
+  </si>
+  <si>
+    <t>EngCoolantPreheatedState</t>
+  </si>
+  <si>
+    <t>EngVentilationStatus</t>
+  </si>
+  <si>
+    <t>FuelPumpPrimerStatus</t>
+  </si>
+  <si>
+    <t>DieselParticulateFilterLampCmd</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrPssvRgnrtionStatus</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtionStatus</t>
+  </si>
+  <si>
+    <t>DieselParticulateFilterStatus</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdStt</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTI</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTC</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhb_0004</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhb_0003</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTA</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTO</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhb_0002</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhb_0001</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTL</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhb_0000</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTS</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTT</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTP</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTE</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnInhbtdDTV</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrAtmtcActvRgnrtnIntt</t>
+  </si>
+  <si>
+    <t>ExhaustSystemHighTempLampCmd</t>
+  </si>
+  <si>
+    <t>DslPrtcltFltrActvRgnrtnFrcdStts</t>
+  </si>
+  <si>
+    <t>Aftertreatment1ExhaustGasTemp1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslPrtcltFltrInt_0000</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1ExhstGsTmp1PrlmnryFMI</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslPrtcltFltrIntkGsTm</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCatalystTankLevel</t>
+  </si>
+  <si>
+    <t>Aftrtrtment1SCRCatalystTankTemp</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtalystTankLevel2</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystTnkLvlPrlmnr</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DEFTnkLwLvlIndicator</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystRgntTnk1TmpP</t>
+  </si>
+  <si>
+    <t>AftrtrtmntSCROprtrIndcmntSvrity</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtalystTankHeater</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystRgntTnk1HtrP</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCatalystTankLevel_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtment1SCRCatalystTankTemp_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtalystTankLevel2_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystTnkLvlPrlmnr_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DEFTnkLwLvlIndicator_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystRgntTnk1TmpP_1</t>
+  </si>
+  <si>
+    <t>AftrtrtmntSCROprtrIndcmntSvrity_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtalystTankHeater_1</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystRgntTnk1HtrP_1</t>
+  </si>
+  <si>
+    <t>AT1T1I</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRActlDsngRgntQntty</t>
+  </si>
+  <si>
+    <t>Aftertreatment1SCRSystemState</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRActlRgntQnttyOfInt</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRDsngRgentAbsPress</t>
+  </si>
+  <si>
+    <t>A1SCREGT</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystIntkGasTemp</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystIntkGsTmpPrl</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystOtltGasTemp</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1SCRCtlystOtltGsTmpPrl</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslOxdtnCtlystIn_0000</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslOxdtnCtlystOt_0000</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslOxdtnCtlystDffPrss</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslOxdtnCtlystIntkGsT</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslOxdtnCtlystOtltGsT</t>
+  </si>
+  <si>
+    <t>Aftrtrtmnt1DslOxdtnCtlystDf_0000</t>
+  </si>
+  <si>
+    <t>WFI</t>
+  </si>
+  <si>
+    <t>WaterInFuelIndicator</t>
+  </si>
+  <si>
+    <t>EngProtectLampCmd</t>
+  </si>
+  <si>
+    <t>EngAmberWarningLampCmd</t>
+  </si>
+  <si>
+    <t>EngRedStopLampCmd</t>
+  </si>
+  <si>
+    <t>OBDMalfunctionIndicatorLampCmd</t>
+  </si>
+  <si>
+    <t>EngBrakeActiveLampCmd</t>
+  </si>
+  <si>
+    <t>CmprssnBrkEnblSwtchIndctrLmpCmd</t>
+  </si>
+  <si>
+    <t>EngOilPressLowLampCmd</t>
+  </si>
+  <si>
+    <t>EngCoolantTempHighLampCmd</t>
+  </si>
+  <si>
+    <t>EngCoolantLevelLowLampCmd</t>
+  </si>
+  <si>
+    <t>EngIdleManagementActiveLampCmd</t>
+  </si>
+  <si>
+    <t>EngAirFilterRestrictionLampCmd</t>
+  </si>
+  <si>
+    <t>EngFuelFilterRestrictedLampCmd</t>
+  </si>
+  <si>
+    <t>DLCD1</t>
+  </si>
+  <si>
+    <t>EngProtectLampData</t>
+  </si>
+  <si>
+    <t>EngAmberWarningLampData</t>
+  </si>
+  <si>
+    <t>EngRedStopLampData</t>
+  </si>
+  <si>
+    <t>OBDMalfunctionIndicatorLampData</t>
+  </si>
+  <si>
+    <t>EngBrakeActiveLampData</t>
+  </si>
+  <si>
+    <t>CmprssnBrkEnblSwtchIndctrLmpDta</t>
+  </si>
+  <si>
+    <t>EngOilPressLowLampData</t>
+  </si>
+  <si>
+    <t>EngCoolantTempHighLampData</t>
+  </si>
+  <si>
+    <t>EngCoolantLevelLowLampData</t>
+  </si>
+  <si>
+    <t>EngIdleManagementActiveLampData</t>
+  </si>
+  <si>
+    <t>EngAirFilterRestrictionLampData</t>
+  </si>
+  <si>
+    <t>EngFuelFilterRestrictedLampData</t>
+  </si>
+  <si>
+    <t>EngWaitToStartLampData</t>
+  </si>
+  <si>
+    <t>ENGINE SPEED SENSOR INFORMATION</t>
+  </si>
+  <si>
+    <t>0,1,2</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>2,3</t>
+  </si>
+  <si>
+    <t>4,5,6</t>
+  </si>
+  <si>
+    <t>4,5</t>
+  </si>
+  <si>
+    <t>6,7</t>
+  </si>
+  <si>
+    <t>2,3,4</t>
+  </si>
+  <si>
+    <t>5,6,7</t>
   </si>
 </sst>
 </file>
@@ -24520,6 +25057,14 @@
         <v>936</v>
       </c>
     </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D42" s="26">
+        <v>61473</v>
+      </c>
+    </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="36"/>
       <c r="B49" s="36"/>
@@ -24539,406 +25084,3389 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67835F87-8E16-4012-B1FC-4AA8A57E1B78}">
-  <dimension ref="B3:H38"/>
+  <dimension ref="B3:S203"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="2" style="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.140625" style="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2" style="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="26" customWidth="1"/>
+    <col min="10" max="10" width="43.28515625" customWidth="1"/>
+    <col min="11" max="11" width="38.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>871</v>
       </c>
       <c r="C3" t="s">
         <v>974</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>983</v>
       </c>
-      <c r="H3" t="str">
-        <f>_xlfn.CONCAT(B3,C3,":",E3,";")</f>
+      <c r="J3" t="str">
+        <f>IF(C3&lt;&gt;"",_xlfn.CONCAT(C3,";"),"")</f>
+        <v>EngOverrideCtrlMode;</v>
+      </c>
+      <c r="K3" t="str">
+        <f>_xlfn.CONCAT(B3,C3,":",H3,";")</f>
         <v>TSC1EngOverrideCtrlMode:USINT;</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>871</v>
       </c>
       <c r="C4" t="s">
         <v>973</v>
       </c>
-      <c r="E4" t="s">
+      <c r="H4" t="s">
         <v>983</v>
       </c>
-      <c r="H4" t="str">
-        <f t="shared" ref="H4:H12" si="0">_xlfn.CONCAT(B4,C4,":",E4,";")</f>
+      <c r="J4" t="str">
+        <f t="shared" ref="J4:J67" si="0">IF(C4&lt;&gt;"",_xlfn.CONCAT(C4,";"),"")</f>
+        <v>EngRqedSpeedCtrlConditions;</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" ref="K4:K12" si="1">_xlfn.CONCAT(B4,C4,":",H4,";")</f>
         <v>TSC1EngRqedSpeedCtrlConditions:USINT;</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>871</v>
       </c>
       <c r="C5" t="s">
         <v>975</v>
       </c>
-      <c r="E5" t="s">
+      <c r="H5" t="s">
         <v>983</v>
       </c>
-      <c r="H5" t="str">
+      <c r="J5" t="str">
         <f t="shared" si="0"/>
+        <v>OverrideCtrlModePriority;</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1OverrideCtrlModePriority:USINT;</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>871</v>
       </c>
       <c r="C6" t="s">
         <v>976</v>
       </c>
-      <c r="E6" t="s">
+      <c r="H6" t="s">
         <v>984</v>
       </c>
-      <c r="H6" t="str">
+      <c r="J6" t="str">
         <f t="shared" si="0"/>
+        <v>EngRqedSpeed_SpeedLimit;</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1EngRqedSpeed_SpeedLimit:REAL;</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>871</v>
       </c>
       <c r="C7" t="s">
         <v>977</v>
       </c>
-      <c r="E7" t="s">
+      <c r="H7" t="s">
         <v>985</v>
       </c>
-      <c r="H7" t="str">
+      <c r="J7" t="str">
         <f t="shared" si="0"/>
+        <v>EngRqedTorque_TorqueLimit;</v>
+      </c>
+      <c r="K7" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1EngRqedTorque_TorqueLimit:INT;</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>871</v>
       </c>
       <c r="C8" t="s">
         <v>978</v>
       </c>
-      <c r="E8" t="s">
+      <c r="H8" t="s">
         <v>983</v>
       </c>
-      <c r="H8" t="str">
+      <c r="J8" t="str">
         <f t="shared" si="0"/>
+        <v>TransmissionRate;</v>
+      </c>
+      <c r="K8" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1TransmissionRate:USINT;</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>871</v>
       </c>
       <c r="C9" t="s">
         <v>979</v>
       </c>
-      <c r="E9" t="s">
+      <c r="H9" t="s">
         <v>983</v>
       </c>
-      <c r="H9" t="str">
+      <c r="J9" t="str">
         <f t="shared" si="0"/>
+        <v>ControlPurpose;</v>
+      </c>
+      <c r="K9" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1ControlPurpose:USINT;</v>
       </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="P9" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>994</v>
+      </c>
+      <c r="S9" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>871</v>
       </c>
       <c r="C10" t="s">
         <v>980</v>
       </c>
-      <c r="E10" t="s">
+      <c r="H10" t="s">
         <v>984</v>
       </c>
-      <c r="H10" t="str">
+      <c r="J10" t="str">
         <f t="shared" si="0"/>
+        <v>EngineRequestedTorqueHiRes;</v>
+      </c>
+      <c r="K10" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1EngineRequestedTorqueHiRes:REAL;</v>
       </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="P10" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>995</v>
+      </c>
+      <c r="S10" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>871</v>
       </c>
       <c r="C11" t="s">
         <v>981</v>
       </c>
-      <c r="E11" t="s">
+      <c r="H11" t="s">
         <v>983</v>
       </c>
-      <c r="H11" t="str">
+      <c r="J11" t="str">
         <f t="shared" si="0"/>
+        <v>MessageCounter;</v>
+      </c>
+      <c r="K11" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1MessageCounter:USINT;</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="P11" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>996</v>
+      </c>
+      <c r="S11" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>871</v>
       </c>
       <c r="C12" t="s">
         <v>982</v>
       </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>983</v>
       </c>
-      <c r="H12" t="str">
+      <c r="J12" t="str">
         <f t="shared" si="0"/>
+        <v>MessageChecksum;</v>
+      </c>
+      <c r="K12" t="str">
+        <f t="shared" si="1"/>
         <v>TSC1MessageChecksum:USINT;</v>
       </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="P12" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>997</v>
+      </c>
+      <c r="S12" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="J13" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="P13" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>998</v>
+      </c>
+      <c r="S13" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="J14" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="P14" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>999</v>
+      </c>
+      <c r="S14" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>895</v>
       </c>
       <c r="C15" t="s">
         <v>986</v>
       </c>
-      <c r="E15" t="s">
+      <c r="H15" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="J15" t="str">
+        <f t="shared" si="0"/>
+        <v>EngTorqueMode;</v>
+      </c>
+      <c r="P15" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>1000</v>
+      </c>
+      <c r="S15" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>895</v>
       </c>
       <c r="C16" t="s">
         <v>987</v>
       </c>
-      <c r="E16" t="s">
+      <c r="H16" t="s">
         <v>984</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J16" t="str">
+        <f t="shared" si="0"/>
+        <v>ActlEngPrcntTrqueHighResolution;</v>
+      </c>
+      <c r="P16" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>1001</v>
+      </c>
+      <c r="S16" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>895</v>
       </c>
       <c r="C17" t="s">
         <v>988</v>
       </c>
-      <c r="E17" t="s">
+      <c r="H17" t="s">
         <v>985</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J17" t="str">
+        <f t="shared" si="0"/>
+        <v>DriversDemandEngPercentTorque;</v>
+      </c>
+      <c r="P17" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>1002</v>
+      </c>
+      <c r="S17" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>895</v>
       </c>
       <c r="C18" t="s">
         <v>989</v>
       </c>
-      <c r="E18" t="s">
+      <c r="H18" t="s">
         <v>985</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J18" t="str">
+        <f t="shared" si="0"/>
+        <v>ActualEngPercentTorque;</v>
+      </c>
+      <c r="P18" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>1003</v>
+      </c>
+      <c r="S18" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>895</v>
       </c>
       <c r="C19" t="s">
         <v>990</v>
       </c>
-      <c r="E19" t="s">
+      <c r="H19" t="s">
         <v>984</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J19" t="str">
+        <f t="shared" si="0"/>
+        <v>EngSpeed;</v>
+      </c>
+      <c r="P19" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>1004</v>
+      </c>
+      <c r="S19" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>895</v>
       </c>
       <c r="C20" t="s">
         <v>991</v>
       </c>
-      <c r="E20" t="s">
+      <c r="H20" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J20" t="str">
+        <f t="shared" si="0"/>
+        <v>SrcAddrssOfCtrllngDvcFrEngCntrl;</v>
+      </c>
+      <c r="P20" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>1005</v>
+      </c>
+      <c r="S20" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>895</v>
       </c>
       <c r="C21" t="s">
         <v>992</v>
       </c>
-      <c r="E21" t="s">
+      <c r="H21" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J21" t="str">
+        <f t="shared" si="0"/>
+        <v>EngStarterMode;</v>
+      </c>
+      <c r="P21" t="s">
+        <v>564</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>1006</v>
+      </c>
+      <c r="S21" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>895</v>
       </c>
       <c r="C22" t="s">
         <v>993</v>
       </c>
-      <c r="E22" t="s">
+      <c r="H22" t="s">
         <v>985</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J22" t="str">
+        <f t="shared" si="0"/>
+        <v>EngDemandPercentTorque;</v>
+      </c>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="J23" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>958</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1008</v>
+      </c>
+      <c r="H24" t="s">
+        <v>983</v>
+      </c>
+      <c r="J24" t="str">
+        <f t="shared" si="0"/>
+        <v>AccelPedal1LowIdleSwitch;</v>
+      </c>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>958</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1009</v>
+      </c>
+      <c r="H25" t="s">
+        <v>983</v>
+      </c>
+      <c r="J25" t="str">
+        <f t="shared" si="0"/>
+        <v>AccelPedalKickdownSwitch;</v>
+      </c>
+    </row>
+    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>564</v>
+        <v>958</v>
       </c>
       <c r="C26" t="s">
-        <v>994</v>
-      </c>
-      <c r="E26" t="s">
+        <v>1010</v>
+      </c>
+      <c r="H26" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J26" t="str">
+        <f t="shared" si="0"/>
+        <v>RoadSpeedLimitStatus;</v>
+      </c>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>564</v>
+        <v>958</v>
       </c>
       <c r="C27" t="s">
-        <v>995</v>
-      </c>
-      <c r="E27" t="s">
+        <v>1011</v>
+      </c>
+      <c r="H27" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="J27" t="str">
+        <f t="shared" si="0"/>
+        <v>AccelPedal2LowIdleSwitch;</v>
+      </c>
+    </row>
+    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>564</v>
+        <v>958</v>
       </c>
       <c r="C28" t="s">
-        <v>996</v>
-      </c>
-      <c r="E28" t="s">
+        <v>1012</v>
+      </c>
+      <c r="H28" t="s">
+        <v>984</v>
+      </c>
+      <c r="J28" t="str">
+        <f t="shared" si="0"/>
+        <v>AccelPedalPos1;</v>
+      </c>
+    </row>
+    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>958</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1013</v>
+      </c>
+      <c r="H29" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>564</v>
-      </c>
-      <c r="C29" t="s">
-        <v>997</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="J29" t="str">
+        <f t="shared" si="0"/>
+        <v>EngPercentLoadAtCurrentSpeed;</v>
+      </c>
+    </row>
+    <row r="30" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>958</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1014</v>
+      </c>
+      <c r="H30" t="s">
+        <v>984</v>
+      </c>
+      <c r="J30" t="str">
+        <f t="shared" si="0"/>
+        <v>RemoteAccelPedalPos;</v>
+      </c>
+    </row>
+    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>958</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H31" t="s">
+        <v>984</v>
+      </c>
+      <c r="J31" t="str">
+        <f t="shared" si="0"/>
+        <v>AccelPedalPos2;</v>
+      </c>
+    </row>
+    <row r="32" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>958</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1016</v>
+      </c>
+      <c r="H32" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>564</v>
-      </c>
-      <c r="C30" t="s">
-        <v>998</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="J32" t="str">
+        <f t="shared" si="0"/>
+        <v>VhclAccelerationRateLimitStatus;</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>958</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1017</v>
+      </c>
+      <c r="H33" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>564</v>
-      </c>
-      <c r="C31" t="s">
-        <v>999</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="J33" t="str">
+        <f t="shared" si="0"/>
+        <v>MmntryEngMaxPowerEnableFeedback;</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>958</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1018</v>
+      </c>
+      <c r="H34" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>564</v>
-      </c>
-      <c r="C32" t="s">
-        <v>1000</v>
-      </c>
-      <c r="E32" t="s">
+      <c r="J34" t="str">
+        <f t="shared" si="0"/>
+        <v>DPFThermalManagementActive;</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>958</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1019</v>
+      </c>
+      <c r="H35" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>564</v>
-      </c>
-      <c r="C33" t="s">
-        <v>1001</v>
-      </c>
-      <c r="E33" t="s">
+      <c r="J35" t="str">
+        <f t="shared" si="0"/>
+        <v>SCRThermalManagementActive;</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>958</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1020</v>
+      </c>
+      <c r="H36" t="s">
+        <v>984</v>
+      </c>
+      <c r="J36" t="str">
+        <f t="shared" si="0"/>
+        <v>ActlMxAvailableEngPercentTorque;</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>958</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1021</v>
+      </c>
+      <c r="H37" t="s">
+        <v>985</v>
+      </c>
+      <c r="J37" t="str">
+        <f t="shared" si="0"/>
+        <v>EstPumpingPercentTorque;</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J38" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>898</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1022</v>
+      </c>
+      <c r="H39" t="s">
+        <v>985</v>
+      </c>
+      <c r="J39" t="str">
+        <f t="shared" si="0"/>
+        <v>NominalFrictionPercentTorque;</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>898</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1023</v>
+      </c>
+      <c r="H40" t="s">
+        <v>1031</v>
+      </c>
+      <c r="J40" t="str">
+        <f t="shared" si="0"/>
+        <v>EngsDesiredOperatingSpeed;</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>898</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1024</v>
+      </c>
+      <c r="H41" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>564</v>
-      </c>
-      <c r="C34" t="s">
-        <v>1002</v>
-      </c>
-      <c r="E34" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>564</v>
-      </c>
-      <c r="C35" t="s">
-        <v>1003</v>
-      </c>
-      <c r="E35" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>564</v>
-      </c>
-      <c r="C36" t="s">
-        <v>1004</v>
-      </c>
-      <c r="E36" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>564</v>
-      </c>
-      <c r="C37" t="s">
-        <v>1005</v>
-      </c>
-      <c r="E37" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
-        <v>564</v>
-      </c>
-      <c r="C38" t="s">
-        <v>1006</v>
-      </c>
-      <c r="E38" t="s">
-        <v>1007</v>
+      <c r="J41" t="str">
+        <f t="shared" si="0"/>
+        <v>EngsDsrdOprtngSpdAsymmtryAdjstmn;</v>
+      </c>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>898</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1025</v>
+      </c>
+      <c r="H42" t="s">
+        <v>985</v>
+      </c>
+      <c r="J42" t="str">
+        <f t="shared" si="0"/>
+        <v>EstEngPrsticLossesPercentTorque;</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B43" t="s">
+        <v>898</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1026</v>
+      </c>
+      <c r="H43" t="s">
+        <v>984</v>
+      </c>
+      <c r="J43" t="str">
+        <f t="shared" si="0"/>
+        <v>Aftrtratment1ExhaustGasMassFlow;</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>898</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1027</v>
+      </c>
+      <c r="H44" t="s">
+        <v>983</v>
+      </c>
+      <c r="J44" t="str">
+        <f t="shared" si="0"/>
+        <v>Aftertreatment1IntakeDewPoint;</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
+        <v>898</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1028</v>
+      </c>
+      <c r="H45" t="s">
+        <v>983</v>
+      </c>
+      <c r="J45" t="str">
+        <f t="shared" si="0"/>
+        <v>Aftertreatment1ExhaustDewPoint;</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B46" t="s">
+        <v>898</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1029</v>
+      </c>
+      <c r="H46" t="s">
+        <v>983</v>
+      </c>
+      <c r="J46" t="str">
+        <f t="shared" si="0"/>
+        <v>Aftertreatment2IntakeDewPoint;</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>898</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1030</v>
+      </c>
+      <c r="H47" t="s">
+        <v>983</v>
+      </c>
+      <c r="J47" t="str">
+        <f t="shared" si="0"/>
+        <v>Aftertreatment2ExhaustDewPoint;</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J48" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>946</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1032</v>
+      </c>
+      <c r="H49" t="s">
+        <v>984</v>
+      </c>
+      <c r="J49" t="str">
+        <f t="shared" si="0"/>
+        <v>EngTrb1ClcltedTurbineIntakeTemp;</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>946</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1033</v>
+      </c>
+      <c r="H50" t="s">
+        <v>984</v>
+      </c>
+      <c r="J50" t="str">
+        <f t="shared" si="0"/>
+        <v>EngTrb1ClcltedTurbineOutletTemp;</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>946</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1034</v>
+      </c>
+      <c r="H51" t="s">
+        <v>984</v>
+      </c>
+      <c r="J51" t="str">
+        <f t="shared" si="0"/>
+        <v>EngExhstGsRcrculation1ValveCtrl;</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>946</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1035</v>
+      </c>
+      <c r="H52" t="s">
+        <v>983</v>
+      </c>
+      <c r="J52" t="str">
+        <f t="shared" si="0"/>
+        <v>EngVrblGmtryTrbArCtrlShtffValve;</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>946</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1036</v>
+      </c>
+      <c r="H53" t="s">
+        <v>983</v>
+      </c>
+      <c r="J53" t="str">
+        <f t="shared" si="0"/>
+        <v>EngVrableGeometryTurbo1CtrlMode;</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
+        <v>946</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1037</v>
+      </c>
+      <c r="H54" t="s">
+        <v>984</v>
+      </c>
+      <c r="J54" t="str">
+        <f t="shared" si="0"/>
+        <v>EngVrblGometryTurbo1ActuatorPos;</v>
+      </c>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J55" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B56" t="s">
+        <v>900</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1038</v>
+      </c>
+      <c r="H56" t="s">
+        <v>984</v>
+      </c>
+      <c r="J56" t="str">
+        <f t="shared" si="0"/>
+        <v>EngCoolantTemp;</v>
+      </c>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B57" t="s">
+        <v>900</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1039</v>
+      </c>
+      <c r="H57" t="s">
+        <v>985</v>
+      </c>
+      <c r="J57" t="str">
+        <f t="shared" si="0"/>
+        <v>EngFuelTemp1;</v>
+      </c>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>900</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1040</v>
+      </c>
+      <c r="H58" t="s">
+        <v>984</v>
+      </c>
+      <c r="J58" t="str">
+        <f t="shared" si="0"/>
+        <v>EngOilTemp1;</v>
+      </c>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>900</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1041</v>
+      </c>
+      <c r="H59" t="s">
+        <v>984</v>
+      </c>
+      <c r="J59" t="str">
+        <f t="shared" si="0"/>
+        <v>EngTurboOilTemp;</v>
+      </c>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>900</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1042</v>
+      </c>
+      <c r="H60" t="s">
+        <v>985</v>
+      </c>
+      <c r="J60" t="str">
+        <f t="shared" si="0"/>
+        <v>EngIntercoolerTemp;</v>
+      </c>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>900</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1043</v>
+      </c>
+      <c r="H61" t="s">
+        <v>984</v>
+      </c>
+      <c r="J61" t="str">
+        <f t="shared" si="0"/>
+        <v>EngIntercoolerThermostatOpening;</v>
+      </c>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J62" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H63" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J63" t="str">
+        <f t="shared" si="0"/>
+        <v>EngFuelDeliveryPress;</v>
+      </c>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1045</v>
+      </c>
+      <c r="H64" t="s">
+        <v>984</v>
+      </c>
+      <c r="J64" t="str">
+        <f t="shared" si="0"/>
+        <v>EngExCrankcaseBlowbyPress;</v>
+      </c>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H65" t="s">
+        <v>984</v>
+      </c>
+      <c r="J65" t="str">
+        <f t="shared" si="0"/>
+        <v>EngOilLevel;</v>
+      </c>
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1047</v>
+      </c>
+      <c r="H66" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J66" t="str">
+        <f t="shared" si="0"/>
+        <v>EngOilPress;</v>
+      </c>
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1048</v>
+      </c>
+      <c r="H67" t="s">
+        <v>1031</v>
+      </c>
+      <c r="J67" t="str">
+        <f t="shared" si="0"/>
+        <v>EngCrankcasePress;</v>
+      </c>
+    </row>
+    <row r="68" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C68" t="s">
+        <v>1049</v>
+      </c>
+      <c r="H68" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J68" t="str">
+        <f t="shared" ref="J68:J131" si="2">IF(C68&lt;&gt;"",_xlfn.CONCAT(C68,";"),"")</f>
+        <v>EngCoolantPress;</v>
+      </c>
+    </row>
+    <row r="69" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C69" t="s">
+        <v>1050</v>
+      </c>
+      <c r="H69" t="s">
+        <v>984</v>
+      </c>
+      <c r="J69" t="str">
+        <f t="shared" si="2"/>
+        <v>EngCoolantLevel;</v>
+      </c>
+    </row>
+    <row r="70" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J70" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>972</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1053</v>
+      </c>
+      <c r="H71" t="s">
+        <v>1057</v>
+      </c>
+      <c r="J71" t="str">
+        <f t="shared" si="2"/>
+        <v>EngInjectionCtrlPress;</v>
+      </c>
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>972</v>
+      </c>
+      <c r="C72" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H72" t="s">
+        <v>1057</v>
+      </c>
+      <c r="J72" t="str">
+        <f t="shared" si="2"/>
+        <v>EngInjectorMeteringRail1Press;</v>
+      </c>
+    </row>
+    <row r="73" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>972</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1055</v>
+      </c>
+      <c r="H73" t="s">
+        <v>1057</v>
+      </c>
+      <c r="J73" t="str">
+        <f t="shared" si="2"/>
+        <v>EngInjectorTimingRail1Press;</v>
+      </c>
+    </row>
+    <row r="74" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>972</v>
+      </c>
+      <c r="C74" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H74" t="s">
+        <v>1057</v>
+      </c>
+      <c r="J74" t="str">
+        <f t="shared" si="2"/>
+        <v>EngInjectorMeteringRail2Press;</v>
+      </c>
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J75" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>903</v>
+      </c>
+      <c r="C76" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H76" t="s">
+        <v>984</v>
+      </c>
+      <c r="J76" t="str">
+        <f t="shared" si="2"/>
+        <v>EngTripFuel;</v>
+      </c>
+    </row>
+    <row r="77" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>903</v>
+      </c>
+      <c r="C77" t="s">
+        <v>1059</v>
+      </c>
+      <c r="H77" t="s">
+        <v>984</v>
+      </c>
+      <c r="J77" t="str">
+        <f t="shared" si="2"/>
+        <v>EngTotalFuelUsed;</v>
+      </c>
+    </row>
+    <row r="78" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J78" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>930</v>
+      </c>
+      <c r="C79" t="s">
+        <v>1060</v>
+      </c>
+      <c r="H79" t="s">
+        <v>984</v>
+      </c>
+      <c r="J79" t="str">
+        <f t="shared" si="2"/>
+        <v>BarometricPress;</v>
+      </c>
+    </row>
+    <row r="80" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>930</v>
+      </c>
+      <c r="C80" t="s">
+        <v>1061</v>
+      </c>
+      <c r="H80" t="s">
+        <v>984</v>
+      </c>
+      <c r="J80" t="str">
+        <f t="shared" si="2"/>
+        <v>CabInteriorTemp;</v>
+      </c>
+    </row>
+    <row r="81" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>930</v>
+      </c>
+      <c r="C81" t="s">
+        <v>1062</v>
+      </c>
+      <c r="H81" t="s">
+        <v>984</v>
+      </c>
+      <c r="J81" t="str">
+        <f t="shared" si="2"/>
+        <v>AmbientAirTemp;</v>
+      </c>
+    </row>
+    <row r="82" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>930</v>
+      </c>
+      <c r="C82" t="s">
+        <v>1063</v>
+      </c>
+      <c r="H82" t="s">
+        <v>985</v>
+      </c>
+      <c r="J82" t="str">
+        <f t="shared" si="2"/>
+        <v>EngAirIntakeTemp;</v>
+      </c>
+    </row>
+    <row r="83" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>930</v>
+      </c>
+      <c r="C83" t="s">
+        <v>1064</v>
+      </c>
+      <c r="H83" t="s">
+        <v>984</v>
+      </c>
+      <c r="J83" t="str">
+        <f t="shared" si="2"/>
+        <v>RoadSurfaceTemp;</v>
+      </c>
+    </row>
+    <row r="84" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J84" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C85" t="s">
+        <v>1065</v>
+      </c>
+      <c r="H85" t="s">
+        <v>984</v>
+      </c>
+      <c r="J85" t="str">
+        <f t="shared" si="2"/>
+        <v>EngDslPrtclateFilterIntakePress;</v>
+      </c>
+    </row>
+    <row r="86" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C86" t="s">
+        <v>1066</v>
+      </c>
+      <c r="H86" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J86" t="str">
+        <f t="shared" si="2"/>
+        <v>EngIntakeManifold1Press;</v>
+      </c>
+    </row>
+    <row r="87" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B87" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C87" t="s">
+        <v>1067</v>
+      </c>
+      <c r="H87" t="s">
+        <v>985</v>
+      </c>
+      <c r="J87" t="str">
+        <f t="shared" si="2"/>
+        <v>EngIntakeManifold1Temp;</v>
+      </c>
+    </row>
+    <row r="88" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C88" t="s">
+        <v>1068</v>
+      </c>
+      <c r="H88" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J88" t="str">
+        <f t="shared" si="2"/>
+        <v>EngAirIntakePress;</v>
+      </c>
+    </row>
+    <row r="89" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B89" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C89" t="s">
+        <v>1069</v>
+      </c>
+      <c r="H89" t="s">
+        <v>984</v>
+      </c>
+      <c r="J89" t="str">
+        <f t="shared" si="2"/>
+        <v>EngAirFilter1DiffPress;</v>
+      </c>
+    </row>
+    <row r="90" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C90" t="s">
+        <v>1070</v>
+      </c>
+      <c r="H90" t="s">
+        <v>984</v>
+      </c>
+      <c r="J90" t="str">
+        <f t="shared" si="2"/>
+        <v>EngExhaustGasTemp;</v>
+      </c>
+    </row>
+    <row r="91" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B91" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C91" t="s">
+        <v>1071</v>
+      </c>
+      <c r="H91" t="s">
+        <v>984</v>
+      </c>
+      <c r="J91" t="str">
+        <f t="shared" si="2"/>
+        <v>EngCoolantFilterDiffPress;</v>
+      </c>
+    </row>
+    <row r="92" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J92" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B93" t="s">
+        <v>928</v>
+      </c>
+      <c r="C93" t="s">
+        <v>1073</v>
+      </c>
+      <c r="H93" t="s">
+        <v>985</v>
+      </c>
+      <c r="J93" t="str">
+        <f t="shared" si="2"/>
+        <v>NetBatteryCurrent;</v>
+      </c>
+    </row>
+    <row r="94" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B94" t="s">
+        <v>928</v>
+      </c>
+      <c r="C94" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H94" t="s">
+        <v>983</v>
+      </c>
+      <c r="J94" t="str">
+        <f t="shared" si="2"/>
+        <v>AltCurrent;</v>
+      </c>
+    </row>
+    <row r="95" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>928</v>
+      </c>
+      <c r="C95" t="s">
+        <v>1075</v>
+      </c>
+      <c r="H95" t="s">
+        <v>1031</v>
+      </c>
+      <c r="J95" t="str">
+        <f t="shared" si="2"/>
+        <v>ChargingSystemPotential;</v>
+      </c>
+    </row>
+    <row r="96" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B96" t="s">
+        <v>928</v>
+      </c>
+      <c r="C96" t="s">
+        <v>1076</v>
+      </c>
+      <c r="H96" t="s">
+        <v>984</v>
+      </c>
+      <c r="J96" t="str">
+        <f t="shared" si="2"/>
+        <v>BatteryPotential_PowerInput1;</v>
+      </c>
+    </row>
+    <row r="97" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B97" t="s">
+        <v>928</v>
+      </c>
+      <c r="C97" t="s">
+        <v>1077</v>
+      </c>
+      <c r="H97" t="s">
+        <v>984</v>
+      </c>
+      <c r="J97" t="str">
+        <f t="shared" si="2"/>
+        <v>KeyswitchBatteryPotential;</v>
+      </c>
+    </row>
+    <row r="98" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J98" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="99" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B99" t="s">
+        <v>938</v>
+      </c>
+      <c r="C99" t="s">
+        <v>1078</v>
+      </c>
+      <c r="H99" t="s">
+        <v>984</v>
+      </c>
+      <c r="J99" t="str">
+        <f t="shared" si="2"/>
+        <v>EngOilLevelRemoteReservoir;</v>
+      </c>
+    </row>
+    <row r="100" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B100" t="s">
+        <v>938</v>
+      </c>
+      <c r="C100" t="s">
+        <v>1079</v>
+      </c>
+      <c r="H100" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J100" t="str">
+        <f t="shared" si="2"/>
+        <v>EngFuelSupplyPumpIntakePress;</v>
+      </c>
+    </row>
+    <row r="101" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B101" t="s">
+        <v>938</v>
+      </c>
+      <c r="C101" t="s">
+        <v>1080</v>
+      </c>
+      <c r="H101" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J101" t="str">
+        <f t="shared" si="2"/>
+        <v>EngFuelFilterDiffPress;</v>
+      </c>
+    </row>
+    <row r="102" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B102" t="s">
+        <v>938</v>
+      </c>
+      <c r="C102" t="s">
+        <v>1081</v>
+      </c>
+      <c r="H102" t="s">
+        <v>984</v>
+      </c>
+      <c r="J102" t="str">
+        <f t="shared" si="2"/>
+        <v>EngWasteOilReservoirLevel;</v>
+      </c>
+    </row>
+    <row r="103" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B103" t="s">
+        <v>938</v>
+      </c>
+      <c r="C103" t="s">
+        <v>1082</v>
+      </c>
+      <c r="H103" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J103" t="str">
+        <f t="shared" si="2"/>
+        <v>EngOilFilterOutletPress;</v>
+      </c>
+    </row>
+    <row r="104" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B104" t="s">
+        <v>938</v>
+      </c>
+      <c r="C104" t="s">
+        <v>1083</v>
+      </c>
+      <c r="H104" t="s">
+        <v>983</v>
+      </c>
+      <c r="J104" t="str">
+        <f t="shared" si="2"/>
+        <v>EngOilPrimingPumpSwitch;</v>
+      </c>
+    </row>
+    <row r="105" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B105" t="s">
+        <v>938</v>
+      </c>
+      <c r="C105" t="s">
+        <v>1084</v>
+      </c>
+      <c r="H105" t="s">
+        <v>983</v>
+      </c>
+      <c r="J105" t="str">
+        <f t="shared" si="2"/>
+        <v>EngOilPrimingState;</v>
+      </c>
+    </row>
+    <row r="106" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B106" t="s">
+        <v>938</v>
+      </c>
+      <c r="C106" t="s">
+        <v>1085</v>
+      </c>
+      <c r="H106" t="s">
+        <v>983</v>
+      </c>
+      <c r="J106" t="str">
+        <f t="shared" si="2"/>
+        <v>EngOilPreHeatedState;</v>
+      </c>
+    </row>
+    <row r="107" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B107" t="s">
+        <v>938</v>
+      </c>
+      <c r="C107" t="s">
+        <v>1086</v>
+      </c>
+      <c r="H107" t="s">
+        <v>983</v>
+      </c>
+      <c r="J107" t="str">
+        <f t="shared" si="2"/>
+        <v>EngCoolantPreheatedState;</v>
+      </c>
+    </row>
+    <row r="108" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B108" t="s">
+        <v>938</v>
+      </c>
+      <c r="C108" t="s">
+        <v>1087</v>
+      </c>
+      <c r="H108" t="s">
+        <v>983</v>
+      </c>
+      <c r="J108" t="str">
+        <f t="shared" si="2"/>
+        <v>EngVentilationStatus;</v>
+      </c>
+    </row>
+    <row r="109" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B109" t="s">
+        <v>938</v>
+      </c>
+      <c r="C109" t="s">
+        <v>1088</v>
+      </c>
+      <c r="H109" t="s">
+        <v>983</v>
+      </c>
+      <c r="J109" t="str">
+        <f t="shared" si="2"/>
+        <v>FuelPumpPrimerStatus;</v>
+      </c>
+    </row>
+    <row r="110" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="111" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B111" t="s">
+        <v>888</v>
+      </c>
+      <c r="C111" s="33" t="s">
+        <v>1089</v>
+      </c>
+      <c r="D111" s="26">
+        <v>0</v>
+      </c>
+      <c r="E111" s="26" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F111" s="26">
+        <v>0</v>
+      </c>
+      <c r="G111" s="26" t="str">
+        <f>_xlfn.CONCAT(D111+1,",",F111+1)</f>
+        <v>1,1</v>
+      </c>
+      <c r="H111" t="s">
+        <v>983</v>
+      </c>
+      <c r="J111" t="str">
+        <f t="shared" si="2"/>
+        <v>DieselParticulateFilterLampCmd;</v>
+      </c>
+    </row>
+    <row r="112" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
+        <v>888</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D112" s="26">
+        <v>1</v>
+      </c>
+      <c r="E112" s="26" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F112" s="26">
+        <v>0</v>
+      </c>
+      <c r="G112" s="26" t="str">
+        <f t="shared" ref="G112:G133" si="3">_xlfn.CONCAT(D112+1,",",F112+1)</f>
+        <v>2,1</v>
+      </c>
+      <c r="H112" t="s">
+        <v>983</v>
+      </c>
+      <c r="J112" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrPssvRgnrtionStatus;</v>
+      </c>
+    </row>
+    <row r="113" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
+        <v>888</v>
+      </c>
+      <c r="C113" s="33" t="s">
+        <v>1091</v>
+      </c>
+      <c r="D113" s="26">
+        <v>1</v>
+      </c>
+      <c r="E113" s="26" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F113" s="26">
+        <v>2</v>
+      </c>
+      <c r="G113" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>2,3</v>
+      </c>
+      <c r="H113" t="s">
+        <v>983</v>
+      </c>
+      <c r="J113" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtionStatus;</v>
+      </c>
+    </row>
+    <row r="114" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
+        <v>888</v>
+      </c>
+      <c r="C114" s="33" t="s">
+        <v>1092</v>
+      </c>
+      <c r="D114" s="26">
+        <v>1</v>
+      </c>
+      <c r="E114" s="26" t="s">
+        <v>1182</v>
+      </c>
+      <c r="F114" s="26">
+        <v>4</v>
+      </c>
+      <c r="G114" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>2,5</v>
+      </c>
+      <c r="H114" t="s">
+        <v>983</v>
+      </c>
+      <c r="J114" t="str">
+        <f t="shared" si="2"/>
+        <v>DieselParticulateFilterStatus;</v>
+      </c>
+    </row>
+    <row r="115" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B115" t="s">
+        <v>888</v>
+      </c>
+      <c r="C115" t="s">
+        <v>1093</v>
+      </c>
+      <c r="D115" s="26">
+        <v>2</v>
+      </c>
+      <c r="E115" s="26" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F115" s="26">
+        <v>0</v>
+      </c>
+      <c r="G115" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>3,1</v>
+      </c>
+      <c r="H115" t="s">
+        <v>983</v>
+      </c>
+      <c r="J115" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdStt;</v>
+      </c>
+    </row>
+    <row r="116" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B116" t="s">
+        <v>888</v>
+      </c>
+      <c r="C116" s="33" t="s">
+        <v>1094</v>
+      </c>
+      <c r="D116" s="26">
+        <v>2</v>
+      </c>
+      <c r="E116" s="26" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F116" s="26">
+        <v>2</v>
+      </c>
+      <c r="G116" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>3,3</v>
+      </c>
+      <c r="H116" t="s">
+        <v>983</v>
+      </c>
+      <c r="J116" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTI;</v>
+      </c>
+    </row>
+    <row r="117" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B117" t="s">
+        <v>888</v>
+      </c>
+      <c r="C117" t="s">
+        <v>1095</v>
+      </c>
+      <c r="D117" s="26">
+        <v>2</v>
+      </c>
+      <c r="E117" s="26" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F117" s="26">
+        <v>4</v>
+      </c>
+      <c r="G117" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>3,5</v>
+      </c>
+      <c r="H117" t="s">
+        <v>983</v>
+      </c>
+      <c r="J117" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTC;</v>
+      </c>
+    </row>
+    <row r="118" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B118" t="s">
+        <v>888</v>
+      </c>
+      <c r="C118" t="s">
+        <v>1096</v>
+      </c>
+      <c r="D118" s="26">
+        <v>2</v>
+      </c>
+      <c r="E118" s="26" t="s">
+        <v>1184</v>
+      </c>
+      <c r="F118" s="26">
+        <v>6</v>
+      </c>
+      <c r="G118" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>3,7</v>
+      </c>
+      <c r="H118" t="s">
+        <v>983</v>
+      </c>
+      <c r="J118" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhb_0004;</v>
+      </c>
+    </row>
+    <row r="119" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B119" t="s">
+        <v>888</v>
+      </c>
+      <c r="C119" t="s">
+        <v>1097</v>
+      </c>
+      <c r="D119" s="26">
+        <v>3</v>
+      </c>
+      <c r="E119" s="26" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F119" s="26">
+        <v>0</v>
+      </c>
+      <c r="G119" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>4,1</v>
+      </c>
+      <c r="H119" t="s">
+        <v>983</v>
+      </c>
+      <c r="J119" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhb_0003;</v>
+      </c>
+    </row>
+    <row r="120" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B120" t="s">
+        <v>888</v>
+      </c>
+      <c r="C120" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D120" s="26">
+        <v>3</v>
+      </c>
+      <c r="E120" s="26" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F120" s="26">
+        <v>2</v>
+      </c>
+      <c r="G120" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>4,3</v>
+      </c>
+      <c r="H120" t="s">
+        <v>983</v>
+      </c>
+      <c r="J120" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTA;</v>
+      </c>
+    </row>
+    <row r="121" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B121" t="s">
+        <v>888</v>
+      </c>
+      <c r="C121" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D121" s="26">
+        <v>3</v>
+      </c>
+      <c r="E121" s="26" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F121" s="26">
+        <v>4</v>
+      </c>
+      <c r="G121" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>4,5</v>
+      </c>
+      <c r="H121" t="s">
+        <v>983</v>
+      </c>
+      <c r="J121" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTO;</v>
+      </c>
+    </row>
+    <row r="122" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>888</v>
+      </c>
+      <c r="C122" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D122" s="26">
+        <v>3</v>
+      </c>
+      <c r="E122" s="26" t="s">
+        <v>1184</v>
+      </c>
+      <c r="F122" s="26">
+        <v>6</v>
+      </c>
+      <c r="G122" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>4,7</v>
+      </c>
+      <c r="H122" t="s">
+        <v>983</v>
+      </c>
+      <c r="J122" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhb_0002;</v>
+      </c>
+    </row>
+    <row r="123" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B123" t="s">
+        <v>888</v>
+      </c>
+      <c r="C123" t="s">
+        <v>1101</v>
+      </c>
+      <c r="D123" s="26">
+        <v>4</v>
+      </c>
+      <c r="E123" s="26" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F123" s="26">
+        <v>0</v>
+      </c>
+      <c r="G123" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>5,1</v>
+      </c>
+      <c r="H123" t="s">
+        <v>983</v>
+      </c>
+      <c r="J123" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhb_0001;</v>
+      </c>
+    </row>
+    <row r="124" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B124" t="s">
+        <v>888</v>
+      </c>
+      <c r="C124" t="s">
+        <v>1102</v>
+      </c>
+      <c r="D124" s="26">
+        <v>4</v>
+      </c>
+      <c r="E124" s="26" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F124" s="26">
+        <v>2</v>
+      </c>
+      <c r="G124" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>5,3</v>
+      </c>
+      <c r="H124" t="s">
+        <v>983</v>
+      </c>
+      <c r="J124" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTL;</v>
+      </c>
+    </row>
+    <row r="125" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
+        <v>888</v>
+      </c>
+      <c r="C125" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D125" s="26">
+        <v>4</v>
+      </c>
+      <c r="E125" s="26" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F125" s="26">
+        <v>4</v>
+      </c>
+      <c r="G125" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>5,5</v>
+      </c>
+      <c r="H125" t="s">
+        <v>983</v>
+      </c>
+      <c r="J125" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhb_0000;</v>
+      </c>
+    </row>
+    <row r="126" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B126" t="s">
+        <v>888</v>
+      </c>
+      <c r="C126" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D126" s="26">
+        <v>4</v>
+      </c>
+      <c r="E126" s="26" t="s">
+        <v>1184</v>
+      </c>
+      <c r="F126" s="26">
+        <v>6</v>
+      </c>
+      <c r="G126" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>5,7</v>
+      </c>
+      <c r="H126" t="s">
+        <v>983</v>
+      </c>
+      <c r="J126" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTS;</v>
+      </c>
+    </row>
+    <row r="127" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>888</v>
+      </c>
+      <c r="C127" s="33" t="s">
+        <v>1105</v>
+      </c>
+      <c r="D127" s="26">
+        <v>5</v>
+      </c>
+      <c r="E127" s="26" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F127" s="26">
+        <v>0</v>
+      </c>
+      <c r="G127" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>6,1</v>
+      </c>
+      <c r="H127" t="s">
+        <v>983</v>
+      </c>
+      <c r="J127" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTT;</v>
+      </c>
+    </row>
+    <row r="128" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>888</v>
+      </c>
+      <c r="C128" s="33" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D128" s="26">
+        <v>5</v>
+      </c>
+      <c r="E128" s="26" t="s">
+        <v>1181</v>
+      </c>
+      <c r="F128" s="26">
+        <v>2</v>
+      </c>
+      <c r="G128" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>6,3</v>
+      </c>
+      <c r="H128" t="s">
+        <v>983</v>
+      </c>
+      <c r="J128" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTP;</v>
+      </c>
+    </row>
+    <row r="129" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>888</v>
+      </c>
+      <c r="C129" t="s">
+        <v>1107</v>
+      </c>
+      <c r="D129" s="26">
+        <v>5</v>
+      </c>
+      <c r="E129" s="26" t="s">
+        <v>1183</v>
+      </c>
+      <c r="F129" s="26">
+        <v>4</v>
+      </c>
+      <c r="G129" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>6,5</v>
+      </c>
+      <c r="H129" t="s">
+        <v>983</v>
+      </c>
+      <c r="J129" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTE;</v>
+      </c>
+    </row>
+    <row r="130" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B130" t="s">
+        <v>888</v>
+      </c>
+      <c r="C130" t="s">
+        <v>1108</v>
+      </c>
+      <c r="D130" s="26">
+        <v>5</v>
+      </c>
+      <c r="E130" s="26" t="s">
+        <v>1184</v>
+      </c>
+      <c r="F130" s="26">
+        <v>6</v>
+      </c>
+      <c r="G130" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>6,7</v>
+      </c>
+      <c r="H130" t="s">
+        <v>983</v>
+      </c>
+      <c r="J130" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrActvRgnrtnInhbtdDTV;</v>
+      </c>
+    </row>
+    <row r="131" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B131" t="s">
+        <v>888</v>
+      </c>
+      <c r="C131" t="s">
+        <v>1109</v>
+      </c>
+      <c r="D131" s="26">
+        <v>6</v>
+      </c>
+      <c r="E131" s="26" t="s">
+        <v>1180</v>
+      </c>
+      <c r="F131" s="26">
+        <v>0</v>
+      </c>
+      <c r="G131" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>7,1</v>
+      </c>
+      <c r="H131" t="s">
+        <v>983</v>
+      </c>
+      <c r="J131" t="str">
+        <f t="shared" si="2"/>
+        <v>DslPrtcltFltrAtmtcActvRgnrtnIntt;</v>
+      </c>
+    </row>
+    <row r="132" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B132" t="s">
+        <v>888</v>
+      </c>
+      <c r="C132" t="s">
+        <v>1110</v>
+      </c>
+      <c r="D132" s="26">
+        <v>6</v>
+      </c>
+      <c r="E132" s="26" t="s">
+        <v>1185</v>
+      </c>
+      <c r="F132" s="26">
+        <v>2</v>
+      </c>
+      <c r="G132" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>7,3</v>
+      </c>
+      <c r="H132" t="s">
+        <v>983</v>
+      </c>
+      <c r="J132" t="str">
+        <f t="shared" ref="J132:J195" si="4">IF(C132&lt;&gt;"",_xlfn.CONCAT(C132,";"),"")</f>
+        <v>ExhaustSystemHighTempLampCmd;</v>
+      </c>
+    </row>
+    <row r="133" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B133" t="s">
+        <v>888</v>
+      </c>
+      <c r="C133" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D133" s="26">
+        <v>6</v>
+      </c>
+      <c r="E133" s="26" t="s">
+        <v>1186</v>
+      </c>
+      <c r="F133" s="26">
+        <v>5</v>
+      </c>
+      <c r="G133" s="26" t="str">
+        <f t="shared" si="3"/>
+        <v>7,6</v>
+      </c>
+      <c r="H133" t="s">
+        <v>983</v>
+      </c>
+      <c r="J133" t="str">
+        <f t="shared" si="4"/>
+        <v>DslPrtcltFltrActvRgnrtnFrcdStts;</v>
+      </c>
+    </row>
+    <row r="134" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J134" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="135" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B135" t="s">
+        <v>935</v>
+      </c>
+      <c r="C135" t="s">
+        <v>1112</v>
+      </c>
+      <c r="H135" t="s">
+        <v>984</v>
+      </c>
+      <c r="J135" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftertreatment1ExhaustGasTemp1;</v>
+      </c>
+    </row>
+    <row r="136" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B136" t="s">
+        <v>935</v>
+      </c>
+      <c r="C136" t="s">
+        <v>1113</v>
+      </c>
+      <c r="H136" t="s">
+        <v>984</v>
+      </c>
+      <c r="J136" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslPrtcltFltrInt_0000;</v>
+      </c>
+    </row>
+    <row r="137" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B137" t="s">
+        <v>935</v>
+      </c>
+      <c r="C137" t="s">
+        <v>1114</v>
+      </c>
+      <c r="H137" t="s">
+        <v>983</v>
+      </c>
+      <c r="J137" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1ExhstGsTmp1PrlmnryFMI;</v>
+      </c>
+    </row>
+    <row r="138" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B138" t="s">
+        <v>935</v>
+      </c>
+      <c r="C138" t="s">
+        <v>1115</v>
+      </c>
+      <c r="H138" t="s">
+        <v>983</v>
+      </c>
+      <c r="J138" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslPrtcltFltrIntkGsTm;</v>
+      </c>
+    </row>
+    <row r="139" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J139" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="140" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C140" t="s">
+        <v>1116</v>
+      </c>
+      <c r="H140" t="s">
+        <v>984</v>
+      </c>
+      <c r="J140" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCatalystTankLevel;</v>
+      </c>
+    </row>
+    <row r="141" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B141" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C141" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H141" t="s">
+        <v>985</v>
+      </c>
+      <c r="J141" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtment1SCRCatalystTankTemp;</v>
+      </c>
+    </row>
+    <row r="142" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C142" t="s">
+        <v>1118</v>
+      </c>
+      <c r="H142" t="s">
+        <v>984</v>
+      </c>
+      <c r="J142" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtalystTankLevel2;</v>
+      </c>
+    </row>
+    <row r="143" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B143" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C143" t="s">
+        <v>1119</v>
+      </c>
+      <c r="H143" t="s">
+        <v>983</v>
+      </c>
+      <c r="J143" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystTnkLvlPrlmnr;</v>
+      </c>
+    </row>
+    <row r="144" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B144" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C144" t="s">
+        <v>1120</v>
+      </c>
+      <c r="H144" t="s">
+        <v>983</v>
+      </c>
+      <c r="J144" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DEFTnkLwLvlIndicator;</v>
+      </c>
+    </row>
+    <row r="145" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C145" t="s">
+        <v>1121</v>
+      </c>
+      <c r="H145" t="s">
+        <v>983</v>
+      </c>
+      <c r="J145" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystRgntTnk1TmpP;</v>
+      </c>
+    </row>
+    <row r="146" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B146" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C146" t="s">
+        <v>1122</v>
+      </c>
+      <c r="H146" t="s">
+        <v>983</v>
+      </c>
+      <c r="J146" t="str">
+        <f t="shared" si="4"/>
+        <v>AftrtrtmntSCROprtrIndcmntSvrity;</v>
+      </c>
+    </row>
+    <row r="147" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B147" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C147" t="s">
+        <v>1123</v>
+      </c>
+      <c r="H147" t="s">
+        <v>984</v>
+      </c>
+      <c r="J147" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtalystTankHeater;</v>
+      </c>
+    </row>
+    <row r="148" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B148" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C148" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H148" t="s">
+        <v>983</v>
+      </c>
+      <c r="J148" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystRgntTnk1HtrP;</v>
+      </c>
+    </row>
+    <row r="149" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B149" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C149" t="s">
+        <v>1125</v>
+      </c>
+      <c r="H149" t="s">
+        <v>984</v>
+      </c>
+      <c r="J149" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCatalystTankLevel_1;</v>
+      </c>
+    </row>
+    <row r="150" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B150" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C150" t="s">
+        <v>1126</v>
+      </c>
+      <c r="H150" t="s">
+        <v>985</v>
+      </c>
+      <c r="J150" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtment1SCRCatalystTankTemp_1;</v>
+      </c>
+    </row>
+    <row r="151" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B151" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C151" t="s">
+        <v>1127</v>
+      </c>
+      <c r="H151" t="s">
+        <v>984</v>
+      </c>
+      <c r="J151" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtalystTankLevel2_1;</v>
+      </c>
+    </row>
+    <row r="152" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B152" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C152" t="s">
+        <v>1128</v>
+      </c>
+      <c r="H152" t="s">
+        <v>983</v>
+      </c>
+      <c r="J152" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystTnkLvlPrlmnr_1;</v>
+      </c>
+    </row>
+    <row r="153" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B153" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C153" t="s">
+        <v>1129</v>
+      </c>
+      <c r="H153" t="s">
+        <v>983</v>
+      </c>
+      <c r="J153" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DEFTnkLwLvlIndicator_1;</v>
+      </c>
+    </row>
+    <row r="154" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B154" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C154" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H154" t="s">
+        <v>983</v>
+      </c>
+      <c r="J154" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystRgntTnk1TmpP_1;</v>
+      </c>
+    </row>
+    <row r="155" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B155" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C155" t="s">
+        <v>1131</v>
+      </c>
+      <c r="H155" t="s">
+        <v>983</v>
+      </c>
+      <c r="J155" t="str">
+        <f t="shared" si="4"/>
+        <v>AftrtrtmntSCROprtrIndcmntSvrity_1;</v>
+      </c>
+    </row>
+    <row r="156" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B156" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C156" t="s">
+        <v>1132</v>
+      </c>
+      <c r="H156" t="s">
+        <v>984</v>
+      </c>
+      <c r="J156" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtalystTankHeater_1;</v>
+      </c>
+    </row>
+    <row r="157" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B157" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C157" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H157" t="s">
+        <v>983</v>
+      </c>
+      <c r="J157" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystRgntTnk1HtrP_1;</v>
+      </c>
+    </row>
+    <row r="158" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J158" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="159" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B159" t="s">
+        <v>940</v>
+      </c>
+      <c r="C159" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H159" t="s">
+        <v>984</v>
+      </c>
+      <c r="J159" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRActlDsngRgntQntty;</v>
+      </c>
+    </row>
+    <row r="160" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B160" t="s">
+        <v>940</v>
+      </c>
+      <c r="C160" t="s">
+        <v>1136</v>
+      </c>
+      <c r="H160" t="s">
+        <v>983</v>
+      </c>
+      <c r="J160" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftertreatment1SCRSystemState;</v>
+      </c>
+    </row>
+    <row r="161" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B161" t="s">
+        <v>940</v>
+      </c>
+      <c r="C161" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H161" t="s">
+        <v>984</v>
+      </c>
+      <c r="J161" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRActlRgntQnttyOfInt;</v>
+      </c>
+    </row>
+    <row r="162" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B162" t="s">
+        <v>940</v>
+      </c>
+      <c r="C162" t="s">
+        <v>1138</v>
+      </c>
+      <c r="H162" t="s">
+        <v>1051</v>
+      </c>
+      <c r="J162" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRDsngRgentAbsPress;</v>
+      </c>
+    </row>
+    <row r="163" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J163" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="164" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B164" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C164" t="s">
+        <v>1140</v>
+      </c>
+      <c r="H164" t="s">
+        <v>984</v>
+      </c>
+      <c r="J164" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystIntkGasTemp;</v>
+      </c>
+    </row>
+    <row r="165" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B165" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C165" t="s">
+        <v>1141</v>
+      </c>
+      <c r="H165" t="s">
+        <v>983</v>
+      </c>
+      <c r="J165" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystIntkGsTmpPrl;</v>
+      </c>
+    </row>
+    <row r="166" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B166" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C166" t="s">
+        <v>1142</v>
+      </c>
+      <c r="H166" t="s">
+        <v>984</v>
+      </c>
+      <c r="J166" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystOtltGasTemp;</v>
+      </c>
+    </row>
+    <row r="167" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B167" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C167" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H167" t="s">
+        <v>983</v>
+      </c>
+      <c r="J167" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1SCRCtlystOtltGsTmpPrl;</v>
+      </c>
+    </row>
+    <row r="168" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J168" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="169" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B169" t="s">
+        <v>950</v>
+      </c>
+      <c r="C169" t="s">
+        <v>1144</v>
+      </c>
+      <c r="H169" t="s">
+        <v>984</v>
+      </c>
+      <c r="J169" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslOxdtnCtlystIn_0000;</v>
+      </c>
+    </row>
+    <row r="170" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B170" t="s">
+        <v>950</v>
+      </c>
+      <c r="C170" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H170" t="s">
+        <v>984</v>
+      </c>
+      <c r="J170" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslOxdtnCtlystOt_0000;</v>
+      </c>
+    </row>
+    <row r="171" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B171" t="s">
+        <v>950</v>
+      </c>
+      <c r="C171" t="s">
+        <v>1146</v>
+      </c>
+      <c r="H171" t="s">
+        <v>984</v>
+      </c>
+      <c r="J171" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslOxdtnCtlystDffPrss;</v>
+      </c>
+    </row>
+    <row r="172" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B172" t="s">
+        <v>950</v>
+      </c>
+      <c r="C172" t="s">
+        <v>1147</v>
+      </c>
+      <c r="H172" t="s">
+        <v>983</v>
+      </c>
+      <c r="J172" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslOxdtnCtlystIntkGsT;</v>
+      </c>
+    </row>
+    <row r="173" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B173" t="s">
+        <v>950</v>
+      </c>
+      <c r="C173" t="s">
+        <v>1148</v>
+      </c>
+      <c r="H173" t="s">
+        <v>983</v>
+      </c>
+      <c r="J173" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslOxdtnCtlystOtltGsT;</v>
+      </c>
+    </row>
+    <row r="174" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B174" t="s">
+        <v>950</v>
+      </c>
+      <c r="C174" t="s">
+        <v>1149</v>
+      </c>
+      <c r="H174" t="s">
+        <v>983</v>
+      </c>
+      <c r="J174" t="str">
+        <f t="shared" si="4"/>
+        <v>Aftrtrtmnt1DslOxdtnCtlystDf_0000;</v>
+      </c>
+    </row>
+    <row r="175" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J175" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="176" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B176" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C176" t="s">
+        <v>1151</v>
+      </c>
+      <c r="H176" t="s">
+        <v>983</v>
+      </c>
+      <c r="J176" t="str">
+        <f t="shared" si="4"/>
+        <v>WaterInFuelIndicator;</v>
+      </c>
+    </row>
+    <row r="177" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J177" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="178" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B178" t="s">
+        <v>961</v>
+      </c>
+      <c r="C178" t="s">
+        <v>1152</v>
+      </c>
+      <c r="H178" t="s">
+        <v>983</v>
+      </c>
+      <c r="I178">
+        <v>1</v>
+      </c>
+      <c r="J178" t="str">
+        <f t="shared" si="4"/>
+        <v>EngProtectLampCmd;</v>
+      </c>
+    </row>
+    <row r="179" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B179" t="s">
+        <v>961</v>
+      </c>
+      <c r="C179" t="s">
+        <v>1153</v>
+      </c>
+      <c r="H179" t="s">
+        <v>983</v>
+      </c>
+      <c r="I179">
+        <v>2</v>
+      </c>
+      <c r="J179" t="str">
+        <f t="shared" si="4"/>
+        <v>EngAmberWarningLampCmd;</v>
+      </c>
+    </row>
+    <row r="180" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B180" t="s">
+        <v>961</v>
+      </c>
+      <c r="C180" t="s">
+        <v>1154</v>
+      </c>
+      <c r="H180" t="s">
+        <v>983</v>
+      </c>
+      <c r="I180">
+        <v>3</v>
+      </c>
+      <c r="J180" t="str">
+        <f t="shared" si="4"/>
+        <v>EngRedStopLampCmd;</v>
+      </c>
+    </row>
+    <row r="181" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B181" t="s">
+        <v>961</v>
+      </c>
+      <c r="C181" t="s">
+        <v>1155</v>
+      </c>
+      <c r="H181" t="s">
+        <v>983</v>
+      </c>
+      <c r="I181">
+        <v>4</v>
+      </c>
+      <c r="J181" t="str">
+        <f t="shared" si="4"/>
+        <v>OBDMalfunctionIndicatorLampCmd;</v>
+      </c>
+    </row>
+    <row r="182" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B182" t="s">
+        <v>961</v>
+      </c>
+      <c r="C182" t="s">
+        <v>1156</v>
+      </c>
+      <c r="H182" t="s">
+        <v>983</v>
+      </c>
+      <c r="I182">
+        <v>5</v>
+      </c>
+      <c r="J182" t="str">
+        <f t="shared" si="4"/>
+        <v>EngBrakeActiveLampCmd;</v>
+      </c>
+    </row>
+    <row r="183" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B183" t="s">
+        <v>961</v>
+      </c>
+      <c r="C183" t="s">
+        <v>1157</v>
+      </c>
+      <c r="H183" t="s">
+        <v>983</v>
+      </c>
+      <c r="I183">
+        <v>6</v>
+      </c>
+      <c r="J183" t="str">
+        <f t="shared" si="4"/>
+        <v>CmprssnBrkEnblSwtchIndctrLmpCmd;</v>
+      </c>
+    </row>
+    <row r="184" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B184" t="s">
+        <v>961</v>
+      </c>
+      <c r="C184" t="s">
+        <v>1158</v>
+      </c>
+      <c r="H184" t="s">
+        <v>983</v>
+      </c>
+      <c r="I184">
+        <v>7</v>
+      </c>
+      <c r="J184" t="str">
+        <f t="shared" si="4"/>
+        <v>EngOilPressLowLampCmd;</v>
+      </c>
+    </row>
+    <row r="185" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B185" t="s">
+        <v>961</v>
+      </c>
+      <c r="C185" t="s">
+        <v>1159</v>
+      </c>
+      <c r="H185" t="s">
+        <v>983</v>
+      </c>
+      <c r="I185">
+        <v>8</v>
+      </c>
+      <c r="J185" t="str">
+        <f t="shared" si="4"/>
+        <v>EngCoolantTempHighLampCmd;</v>
+      </c>
+    </row>
+    <row r="186" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B186" t="s">
+        <v>961</v>
+      </c>
+      <c r="C186" t="s">
+        <v>1160</v>
+      </c>
+      <c r="H186" t="s">
+        <v>983</v>
+      </c>
+      <c r="I186">
+        <v>9</v>
+      </c>
+      <c r="J186" t="str">
+        <f t="shared" si="4"/>
+        <v>EngCoolantLevelLowLampCmd;</v>
+      </c>
+    </row>
+    <row r="187" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B187" t="s">
+        <v>961</v>
+      </c>
+      <c r="C187" t="s">
+        <v>1161</v>
+      </c>
+      <c r="H187" t="s">
+        <v>983</v>
+      </c>
+      <c r="I187">
+        <v>10</v>
+      </c>
+      <c r="J187" t="str">
+        <f t="shared" si="4"/>
+        <v>EngIdleManagementActiveLampCmd;</v>
+      </c>
+    </row>
+    <row r="188" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B188" t="s">
+        <v>961</v>
+      </c>
+      <c r="C188" t="s">
+        <v>1162</v>
+      </c>
+      <c r="H188" t="s">
+        <v>983</v>
+      </c>
+      <c r="I188">
+        <v>11</v>
+      </c>
+      <c r="J188" t="str">
+        <f t="shared" si="4"/>
+        <v>EngAirFilterRestrictionLampCmd;</v>
+      </c>
+    </row>
+    <row r="189" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B189" t="s">
+        <v>961</v>
+      </c>
+      <c r="C189" t="s">
+        <v>1163</v>
+      </c>
+      <c r="H189" t="s">
+        <v>983</v>
+      </c>
+      <c r="I189">
+        <v>12</v>
+      </c>
+      <c r="J189" t="str">
+        <f t="shared" si="4"/>
+        <v>EngFuelFilterRestrictedLampCmd;</v>
+      </c>
+    </row>
+    <row r="190" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J190" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+    </row>
+    <row r="191" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B191" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C191" t="s">
+        <v>1165</v>
+      </c>
+      <c r="H191" t="s">
+        <v>983</v>
+      </c>
+      <c r="I191">
+        <v>1</v>
+      </c>
+      <c r="J191" t="str">
+        <f t="shared" si="4"/>
+        <v>EngProtectLampData;</v>
+      </c>
+    </row>
+    <row r="192" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B192" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C192" t="s">
+        <v>1166</v>
+      </c>
+      <c r="H192" t="s">
+        <v>983</v>
+      </c>
+      <c r="I192">
+        <v>2</v>
+      </c>
+      <c r="J192" t="str">
+        <f t="shared" si="4"/>
+        <v>EngAmberWarningLampData;</v>
+      </c>
+    </row>
+    <row r="193" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B193" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C193" t="s">
+        <v>1167</v>
+      </c>
+      <c r="H193" t="s">
+        <v>983</v>
+      </c>
+      <c r="I193">
+        <v>3</v>
+      </c>
+      <c r="J193" t="str">
+        <f t="shared" si="4"/>
+        <v>EngRedStopLampData;</v>
+      </c>
+    </row>
+    <row r="194" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B194" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C194" t="s">
+        <v>1168</v>
+      </c>
+      <c r="H194" t="s">
+        <v>983</v>
+      </c>
+      <c r="I194">
+        <v>4</v>
+      </c>
+      <c r="J194" t="str">
+        <f t="shared" si="4"/>
+        <v>OBDMalfunctionIndicatorLampData;</v>
+      </c>
+    </row>
+    <row r="195" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B195" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C195" t="s">
+        <v>1169</v>
+      </c>
+      <c r="H195" t="s">
+        <v>983</v>
+      </c>
+      <c r="I195">
+        <v>5</v>
+      </c>
+      <c r="J195" t="str">
+        <f t="shared" si="4"/>
+        <v>EngBrakeActiveLampData;</v>
+      </c>
+    </row>
+    <row r="196" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B196" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C196" t="s">
+        <v>1170</v>
+      </c>
+      <c r="H196" t="s">
+        <v>983</v>
+      </c>
+      <c r="I196">
+        <v>6</v>
+      </c>
+      <c r="J196" t="str">
+        <f t="shared" ref="J196:J203" si="5">IF(C196&lt;&gt;"",_xlfn.CONCAT(C196,";"),"")</f>
+        <v>CmprssnBrkEnblSwtchIndctrLmpDta;</v>
+      </c>
+    </row>
+    <row r="197" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B197" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C197" t="s">
+        <v>1171</v>
+      </c>
+      <c r="H197" t="s">
+        <v>983</v>
+      </c>
+      <c r="I197">
+        <v>7</v>
+      </c>
+      <c r="J197" t="str">
+        <f t="shared" si="5"/>
+        <v>EngOilPressLowLampData;</v>
+      </c>
+    </row>
+    <row r="198" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B198" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C198" t="s">
+        <v>1172</v>
+      </c>
+      <c r="H198" t="s">
+        <v>983</v>
+      </c>
+      <c r="I198">
+        <v>8</v>
+      </c>
+      <c r="J198" t="str">
+        <f t="shared" si="5"/>
+        <v>EngCoolantTempHighLampData;</v>
+      </c>
+    </row>
+    <row r="199" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B199" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C199" t="s">
+        <v>1173</v>
+      </c>
+      <c r="H199" t="s">
+        <v>983</v>
+      </c>
+      <c r="I199">
+        <v>9</v>
+      </c>
+      <c r="J199" t="str">
+        <f t="shared" si="5"/>
+        <v>EngCoolantLevelLowLampData;</v>
+      </c>
+    </row>
+    <row r="200" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B200" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C200" t="s">
+        <v>1174</v>
+      </c>
+      <c r="H200" t="s">
+        <v>983</v>
+      </c>
+      <c r="I200">
+        <v>10</v>
+      </c>
+      <c r="J200" t="str">
+        <f t="shared" si="5"/>
+        <v>EngIdleManagementActiveLampData;</v>
+      </c>
+    </row>
+    <row r="201" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B201" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C201" t="s">
+        <v>1175</v>
+      </c>
+      <c r="H201" t="s">
+        <v>983</v>
+      </c>
+      <c r="I201">
+        <v>11</v>
+      </c>
+      <c r="J201" t="str">
+        <f t="shared" si="5"/>
+        <v>EngAirFilterRestrictionLampData;</v>
+      </c>
+    </row>
+    <row r="202" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B202" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1176</v>
+      </c>
+      <c r="H202" t="s">
+        <v>983</v>
+      </c>
+      <c r="I202">
+        <v>12</v>
+      </c>
+      <c r="J202" t="str">
+        <f t="shared" si="5"/>
+        <v>EngFuelFilterRestrictedLampData;</v>
+      </c>
+    </row>
+    <row r="203" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B203" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C203" t="s">
+        <v>1177</v>
+      </c>
+      <c r="H203" t="s">
+        <v>983</v>
+      </c>
+      <c r="I203">
+        <v>13</v>
+      </c>
+      <c r="J203" t="str">
+        <f t="shared" si="5"/>
+        <v>EngWaitToStartLampData;</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c96d9849-7071-4555-8535-ee11c374d0f7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef" xsi:nil="true"/>
+    <SharedWithUsers xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef">
+      <UserInfo>
+        <DisplayName>Noel Loughran</DisplayName>
+        <AccountId>19</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25165,27 +28693,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c96d9849-7071-4555-8535-ee11c374d0f7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef" xsi:nil="true"/>
-    <SharedWithUsers xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef">
-      <UserInfo>
-        <DisplayName>Noel Loughran</DisplayName>
-        <AccountId>19</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DE4EA8D-9182-4C6A-B31C-49373749A7AE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="3f324c86-ae15-4ed4-b4a2-09335a7d28ef"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="c96d9849-7071-4555-8535-ee11c374d0f7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -25210,18 +28738,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DE4EA8D-9182-4C6A-B31C-49373749A7AE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="3f324c86-ae15-4ed4-b4a2-09335a7d28ef"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="c96d9849-7071-4555-8535-ee11c374d0f7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
EXCEL for the last Commit
</commit_message>
<xml_diff>
--- a/T620X_IO.xlsx
+++ b/T620X_IO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev_plc\MTech\MTech_T620X_Trommel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49464D75-6129-474D-9E3A-402C8D09734C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE95135-CF38-414E-8EEB-23CC7FBCAA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15720" tabRatio="857" activeTab="7" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
+    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15720" tabRatio="857" activeTab="9" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
   </bookViews>
   <sheets>
     <sheet name="IO" sheetId="11" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="ALARMS" sheetId="24" r:id="rId5"/>
     <sheet name="ALARMS_IO" sheetId="31" r:id="rId6"/>
     <sheet name="SNAGS" sheetId="33" r:id="rId7"/>
-    <sheet name="Sheet2" sheetId="37" r:id="rId8"/>
+    <sheet name="DPF Symbol Logic" sheetId="37" r:id="rId8"/>
     <sheet name="  C3.6 PGNs" sheetId="35" r:id="rId9"/>
     <sheet name="C3.6 PGNS -12 doc" sheetId="36" r:id="rId10"/>
   </sheets>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3144" uniqueCount="1186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3150" uniqueCount="1188">
   <si>
     <t>PLC Name</t>
   </si>
@@ -3609,6 +3609,12 @@
   </si>
   <si>
     <t>GVL_Engine.MILamp=FALSE</t>
+  </si>
+  <si>
+    <t>Engine hours  request</t>
+  </si>
+  <si>
+    <t>Method for setting speed a bit random ….?</t>
   </si>
 </sst>
 </file>
@@ -10753,7 +10759,7 @@
     <col min="7" max="7" width="5.140625" style="26" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="2" style="26" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.140625" style="26" customWidth="1"/>
-    <col min="12" max="12" width="43.28515625" customWidth="1"/>
+    <col min="12" max="12" width="43.28515625" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="50.28515625" customWidth="1"/>
     <col min="14" max="14" width="44" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="49" bestFit="1" customWidth="1"/>
@@ -12444,7 +12450,7 @@
         <v>682</v>
       </c>
       <c r="J49" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="L49" t="str">
         <f t="shared" si="0"/>
@@ -12460,7 +12466,7 @@
       </c>
       <c r="O49" t="str">
         <f t="shared" si="3"/>
-        <v>ET1_EngCoolantTemp:REAL; // SPN:1637</v>
+        <v>ET1_EngCoolantTemp:INT; // SPN:1637</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
@@ -13822,7 +13828,7 @@
         <v>EFS_EngOilFilterOutletPress:UINT; // SPN:3549</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -13834,9 +13840,6 @@
       </c>
       <c r="D90" s="35">
         <v>3550</v>
-      </c>
-      <c r="E90" t="s">
-        <v>682</v>
       </c>
       <c r="J90" t="s">
         <v>983</v>
@@ -13858,7 +13861,7 @@
         <v>EFS_EngOilPrimingPumpSwitch:USINT; // SPN:3550</v>
       </c>
     </row>
-    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -13870,6 +13873,9 @@
       </c>
       <c r="D91" s="35">
         <v>3551</v>
+      </c>
+      <c r="E91" t="s">
+        <v>682</v>
       </c>
       <c r="J91" t="s">
         <v>983</v>
@@ -31089,6 +31095,9 @@
       <c r="C90" t="s">
         <v>865</v>
       </c>
+      <c r="D90" t="s">
+        <v>589</v>
+      </c>
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
@@ -31112,6 +31121,25 @@
       </c>
       <c r="C93" t="s">
         <v>864</v>
+      </c>
+    </row>
+    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B95" t="s">
+        <v>669</v>
+      </c>
+      <c r="C95" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D95" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="96" spans="2:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B96" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C96" s="33" t="s">
+        <v>1187</v>
       </c>
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.25">
@@ -31982,33 +32010,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c96d9849-7071-4555-8535-ee11c374d0f7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef" xsi:nil="true"/>
-    <SharedWithUsers xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef">
-      <UserInfo>
-        <DisplayName>Noel Loughran</DisplayName>
-        <AccountId>19</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007A9F7729ADF49144A01A6175DD599202" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3f00ebe7287476f312414df31db46304">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c96d9849-7071-4555-8535-ee11c374d0f7" xmlns:ns3="3f324c86-ae15-4ed4-b4a2-09335a7d28ef" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8f2e969a0d0c60cbdf6bd0d859a86451" ns2:_="" ns3:_="">
     <xsd:import namespace="c96d9849-7071-4555-8535-ee11c374d0f7"/>
@@ -32231,32 +32232,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DE4EA8D-9182-4C6A-B31C-49373749A7AE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="3f324c86-ae15-4ed4-b4a2-09335a7d28ef"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="c96d9849-7071-4555-8535-ee11c374d0f7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c96d9849-7071-4555-8535-ee11c374d0f7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef" xsi:nil="true"/>
+    <SharedWithUsers xmlns="3f324c86-ae15-4ed4-b4a2-09335a7d28ef">
+      <UserInfo>
+        <DisplayName>Noel Loughran</DisplayName>
+        <AccountId>19</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6596B7D1-B3E6-40CB-B05E-2E959D1A2B6D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -32273,4 +32276,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DE4EA8D-9182-4C6A-B31C-49373749A7AE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="3f324c86-ae15-4ed4-b4a2-09335a7d28ef"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="c96d9849-7071-4555-8535-ee11c374d0f7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
MIMIC swapped in the new isometric images, Radial mode up and going Radial Mode - manual mode - changed over 2 + 3 to match the auto sequence start up
</commit_message>
<xml_diff>
--- a/T620X_IO.xlsx
+++ b/T620X_IO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev_plc\MTech\MTech_T620X_Trommel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709D9869-B1E7-44F9-A3DD-A3FA48B7EEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09B68600-DA9A-48D9-AF99-48653C91BDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15720" tabRatio="857" activeTab="7" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
+    <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15720" tabRatio="857" activeTab="4" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
   </bookViews>
   <sheets>
     <sheet name="IO" sheetId="11" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2686" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2687" uniqueCount="937">
   <si>
     <t>PLC Name</t>
   </si>
@@ -2857,6 +2857,9 @@
   </si>
   <si>
     <t>Hydraulic Oil level Low Alarm</t>
+  </si>
+  <si>
+    <t>CollectConveyor_RectIcon_FB.Fill_Colour</t>
   </si>
 </sst>
 </file>
@@ -18049,7 +18052,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A526D88A-D53C-48FF-978F-7E496FB8AA8D}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:E131"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -18073,7 +18075,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -18087,7 +18089,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -18101,7 +18103,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -18115,7 +18117,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -18129,7 +18131,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -18146,7 +18148,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -18160,7 +18162,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -18174,7 +18176,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -18188,7 +18190,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -18202,7 +18204,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -18216,7 +18218,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -18230,7 +18232,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -18244,7 +18246,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -18258,7 +18260,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -18272,7 +18274,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -18286,7 +18288,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -18300,7 +18302,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -18314,7 +18316,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -18331,7 +18333,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -18345,7 +18347,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -18359,7 +18361,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -18373,7 +18375,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -18390,7 +18392,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -18404,7 +18406,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -18418,7 +18420,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -18432,7 +18434,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -18446,7 +18448,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -18463,7 +18465,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -18491,7 +18493,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -18508,7 +18510,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -18522,7 +18524,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -18539,7 +18541,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -18556,7 +18558,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -18573,7 +18575,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -18587,7 +18589,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -18601,7 +18603,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -18615,7 +18617,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -18632,7 +18634,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -18649,7 +18651,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -18663,7 +18665,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -18691,7 +18693,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -18705,7 +18707,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -18722,7 +18724,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -18736,7 +18738,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -18750,7 +18752,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -18764,7 +18766,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -18778,7 +18780,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -18795,7 +18797,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -18809,7 +18811,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -18826,7 +18828,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -18840,7 +18842,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -18854,7 +18856,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -18868,7 +18870,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -18893,7 +18895,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -18907,7 +18909,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -18924,7 +18926,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -18938,7 +18940,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -18952,7 +18954,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -18966,7 +18968,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -18997,7 +18999,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -19028,7 +19030,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -19045,7 +19047,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -19059,7 +19061,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>69</v>
       </c>
@@ -19076,7 +19078,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>70</v>
       </c>
@@ -19090,7 +19092,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>71</v>
       </c>
@@ -19134,8 +19136,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>570</v>
       </c>
@@ -19154,8 +19155,6 @@
         <v>567</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
         <v>552</v>
@@ -19175,8 +19174,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="82" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>555</v>
       </c>
@@ -19187,7 +19185,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="84" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C84" t="s">
         <v>579</v>
       </c>
@@ -19198,8 +19196,6 @@
         <v>580</v>
       </c>
     </row>
-    <row r="85" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="87" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>288</v>
@@ -19208,7 +19204,6 @@
         <v>581</v>
       </c>
     </row>
-    <row r="88" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="89" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>570</v>
@@ -19217,7 +19212,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="90" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>288</v>
       </c>
@@ -19228,7 +19223,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="91" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>288</v>
       </c>
@@ -19255,8 +19250,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="94" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>390</v>
       </c>
@@ -19275,17 +19269,11 @@
         <v>908</v>
       </c>
     </row>
-    <row r="97" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="E102" t="s">
+        <v>936</v>
+      </c>
+    </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>555</v>
@@ -19294,8 +19282,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="109" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C110" t="s">
         <v>558</v>
       </c>
@@ -19316,7 +19303,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="113" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C113" t="s">
         <v>560</v>
       </c>
@@ -19324,7 +19311,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="114" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C114" t="s">
         <v>563</v>
       </c>
@@ -19332,7 +19319,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="115" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C115" t="s">
         <v>561</v>
       </c>
@@ -19340,9 +19327,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="116" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C118" t="s">
         <v>558</v>
       </c>
@@ -19363,7 +19348,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="121" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C121" t="s">
         <v>560</v>
       </c>
@@ -19371,7 +19356,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="122" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C122" t="s">
         <v>563</v>
       </c>
@@ -19379,7 +19364,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="123" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C123" t="s">
         <v>561</v>
       </c>
@@ -19387,10 +19372,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="124" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="2:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B127">
         <v>1</v>
       </c>
@@ -19412,7 +19394,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="129" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B129">
         <v>3</v>
       </c>
@@ -19423,7 +19405,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="130" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B130">
         <v>4</v>
       </c>
@@ -19434,7 +19416,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="131" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B131">
         <v>5</v>
       </c>
@@ -19446,16 +19428,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E131" xr:uid="{A526D88A-D53C-48FF-978F-7E496FB8AA8D}">
-    <filterColumn colId="2">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -26830,6 +26802,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c96d9849-7071-4555-8535-ee11c374d0f7">
@@ -26845,15 +26826,6 @@
     </SharedWithUsers>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -26876,6 +26848,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DE4EA8D-9182-4C6A-B31C-49373749A7AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="3f324c86-ae15-4ed4-b4a2-09335a7d28ef"/>
@@ -26890,12 +26870,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
MIMIC - standard T20X iso view now done
</commit_message>
<xml_diff>
--- a/T620X_IO.xlsx
+++ b/T620X_IO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev_plc\MTech\MTech_T620X_Trommel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B040C4-30AF-46E9-923D-8F0941E25534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00B3BF4-C8BA-42A6-AD44-D4C6D28929F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="5280" windowWidth="29040" windowHeight="15720" tabRatio="857" activeTab="4" xr2:uid="{2FCBBB71-3591-49CF-88C3-9E3184A7626E}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2696" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2698" uniqueCount="940">
   <si>
     <t>PLC Name</t>
   </si>
@@ -2867,6 +2867,9 @@
   </si>
   <si>
     <t>better lines! Show ecu symbol on the engine can link - maybe just schamtic style</t>
+  </si>
+  <si>
+    <t>Better Drum Pressure Display, move counter to interlocks page</t>
   </si>
 </sst>
 </file>
@@ -18228,7 +18231,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A526D88A-D53C-48FF-978F-7E496FB8AA8D}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.42578125" customWidth="1"/>
@@ -19529,6 +19532,14 @@
       </c>
       <c r="E89" s="33" t="s">
         <v>936</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>290</v>
+      </c>
+      <c r="C90" t="s">
+        <v>939</v>
       </c>
     </row>
   </sheetData>
@@ -26706,15 +26717,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007A9F7729ADF49144A01A6175DD599202" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3f00ebe7287476f312414df31db46304">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c96d9849-7071-4555-8535-ee11c374d0f7" xmlns:ns3="3f324c86-ae15-4ed4-b4a2-09335a7d28ef" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8f2e969a0d0c60cbdf6bd0d859a86451" ns2:_="" ns3:_="">
     <xsd:import namespace="c96d9849-7071-4555-8535-ee11c374d0f7"/>
@@ -26937,6 +26939,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DE4EA8D-9182-4C6A-B31C-49373749A7AE}">
   <ds:schemaRefs>
@@ -26955,14 +26966,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6596B7D1-B3E6-40CB-B05E-2E959D1A2B6D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -26979,4 +26982,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3E59E7C-5896-4162-AB70-9CA3CEB6A0FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>